<commit_message>
Clarify Decisao has 8 product rows and bust Excel Online file cache.
Users on an old copy saw empty lines 8-9; grading now explains to reopen the updated pack.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/exercicios/treino-compras-03-decisao.xlsx
+++ b/public/exercicios/treino-compras-03-decisao.xlsx
@@ -13,12 +13,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="28">
   <si>
     <t>TREINO COMPRAS — Exercício 3: Decisão com Empate</t>
   </si>
   <si>
-    <t>Preencha F (TotalA), G (TotalB) e H (Vencedor).</t>
+    <t>Preencha F (TotalA), G (TotalB) e H (Vencedor) nas linhas 2 a 9 (8 produtos).</t>
+  </si>
+  <si>
+    <t>Linha 8 = Óculos proteção | Linha 9 = Abraçadeira</t>
   </si>
   <si>
     <t/>
@@ -617,7 +620,7 @@
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
@@ -637,7 +640,7 @@
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
@@ -696,7 +699,9 @@
       <c r="P9" s="1"/>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A10" s="1"/>
+      <c r="A10" s="1" t="s">
+        <v>8</v>
+      </c>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
@@ -1451,28 +1456,28 @@
   <sheetData>
     <row r="1" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="I1" s="3"/>
       <c r="J1" s="3"/>
@@ -1485,7 +1490,7 @@
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B2" s="1">
         <v>400</v>
@@ -1513,7 +1518,7 @@
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B3" s="1">
         <v>95</v>
@@ -1541,7 +1546,7 @@
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B4" s="1">
         <v>680</v>
@@ -1569,7 +1574,7 @@
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B5" s="1">
         <v>280</v>
@@ -1597,7 +1602,7 @@
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B6" s="1">
         <v>32</v>
@@ -1625,7 +1630,7 @@
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B7" s="1">
         <v>105</v>
@@ -1653,7 +1658,7 @@
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B8" s="1">
         <v>125</v>
@@ -1681,7 +1686,7 @@
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B9" s="1">
         <v>40</v>
@@ -2458,16 +2463,16 @@
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
@@ -2484,7 +2489,7 @@
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B2" s="1">
         <v>430</v>
@@ -2493,7 +2498,7 @@
         <v>430</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
@@ -2510,7 +2515,7 @@
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B3" s="1">
         <v>120</v>
@@ -2519,7 +2524,7 @@
         <v>110</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
@@ -2536,7 +2541,7 @@
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B4" s="1">
         <v>725</v>
@@ -2545,7 +2550,7 @@
         <v>710</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
@@ -2562,7 +2567,7 @@
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B5" s="1">
         <v>320</v>
@@ -2571,7 +2576,7 @@
         <v>320</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
@@ -2588,7 +2593,7 @@
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B6" s="1">
         <v>60</v>
@@ -2597,7 +2602,7 @@
         <v>64</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E6" s="1"/>
       <c r="F6" s="1"/>
@@ -2614,7 +2619,7 @@
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B7" s="1">
         <v>123</v>
@@ -2623,7 +2628,7 @@
         <v>122.5</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
@@ -2640,7 +2645,7 @@
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B8" s="1">
         <v>145</v>
@@ -2649,7 +2654,7 @@
         <v>145</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E8" s="1"/>
       <c r="F8" s="1"/>
@@ -2666,7 +2671,7 @@
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B9" s="1">
         <v>50</v>
@@ -2675,7 +2680,7 @@
         <v>50</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E9" s="1"/>
       <c r="F9" s="1"/>

</xml_diff>

<commit_message>
Use clearer Empate-first SE formula for Decisao winner column.
The previous nested greater-than form was resolving to Empate whenever B should win; check equality first then A vs B.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/exercicios/treino-compras-03-decisao.xlsx
+++ b/public/exercicios/treino-compras-03-decisao.xlsx
@@ -27,16 +27,16 @@
     <t/>
   </si>
   <si>
-    <t>Fórmula do vencedor (PT-BR):</t>
+    <t>Fórmula do vencedor (PT-BR) — copie exatamente:</t>
   </si>
   <si>
-    <t>=SE(F2&lt;G2;"A";SE(F2&gt;G2;"B";"Empate"))</t>
+    <t>=SE(F2=G2;"Empate";SE(F2&lt;G2;"A";"B"))</t>
   </si>
   <si>
-    <t>Em inglês: =IF(F2&lt;G2,"A",IF(F2&gt;G2,"B","Empate"))</t>
+    <t>Em inglês: =IF(F2=G2,"Empate",IF(F2&lt;G2,"A","B"))</t>
   </si>
   <si>
-    <t>Se TotalA = TotalB, o Excel escreve Empate (não escolhe A nem B).</t>
+    <t>1º: se totais iguais → Empate | 2º: se A menor → A | senão → B</t>
   </si>
   <si>
     <t>Se estiver só visualizando: Editar no navegador / Salvar uma cópia.</t>

</xml_diff>